<commit_message>
cap nhat mon an
</commit_message>
<xml_diff>
--- a/data/danh_sach_mon_an.xlsx
+++ b/data/danh_sach_mon_an.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BTL TRI TUE NHAN TAO\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834E3BF4-7A12-4E6E-A4F0-DA05D7B44753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0423CEB-44E3-4A4F-812E-B2F8FAE9CC70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{83411BAF-91DA-4BCB-8993-1CE8A2F2A6CD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="356">
   <si>
     <t>id</t>
   </si>
@@ -974,12 +974,6 @@
     <t>Gỏi xoài cá sặc</t>
   </si>
   <si>
-    <t>Mùa khô, Mùa mưa</t>
-  </si>
-  <si>
-    <t>Cá</t>
-  </si>
-  <si>
     <t>Gỏi xoài cá sặc, món dân dã miền Nam, nổi bật với hương vị hài hòa, khó cưỡng. Món ăn lý tưởng cho ngày hè nóng nhờ xoài xanh chua giòn và cá sặc khô đậm đà. Nguyên liệu gồm xoài thái sợi, cá nướng thơm, cùng nước mắm tỏi ớt, đường, chanh, rau thơm hòa quyện. Vị chua nhẹ của xoài, mặn béo của cá khô thêm chút cay nơi đầu lưỡi tạo cảm giác khó quên. Đây là món khai vị hấp dẫn và đem lại nét mới mẻ cho bữa cơm gia đình.</t>
   </si>
   <si>
@@ -1025,33 +1019,12 @@
     <t>Thịt</t>
   </si>
   <si>
-    <t>Bột</t>
-  </si>
-  <si>
-    <t>Bánh tằm</t>
-  </si>
-  <si>
-    <t>Hải sản</t>
-  </si>
-  <si>
-    <t>Mùa mưa, Mùa khô</t>
-  </si>
-  <si>
     <t>Quanh năm</t>
   </si>
   <si>
-    <t>Ngọt, Cay, Mặn</t>
-  </si>
-  <si>
-    <t>Chua, Cay, Mặn</t>
-  </si>
-  <si>
     <t>Đắng, Ngọt</t>
   </si>
   <si>
-    <t>Béo, Mặn, Ngọt</t>
-  </si>
-  <si>
     <t>Mặn, Ngọt</t>
   </si>
   <si>
@@ -1073,7 +1046,64 @@
     <t>Béo, Ngot</t>
   </si>
   <si>
-    <t>Mắm, Rau củ quả, Hải sản</t>
+    <t>Chua, Ngọt, Đắng</t>
+  </si>
+  <si>
+    <t>Chua, Cay</t>
+  </si>
+  <si>
+    <t>Mùa mưa</t>
+  </si>
+  <si>
+    <t>Lá giang</t>
+  </si>
+  <si>
+    <t>Cá, Trái cây</t>
+  </si>
+  <si>
+    <t>Mùa khô, Mùa nước nổi</t>
+  </si>
+  <si>
+    <t>Chua, Ngọt, Mặn</t>
+  </si>
+  <si>
+    <t>Cá, Gạo</t>
+  </si>
+  <si>
+    <t>Bột, Trứng</t>
+  </si>
+  <si>
+    <t>Béo, Ngọt</t>
+  </si>
+  <si>
+    <t>Mùa khô</t>
+  </si>
+  <si>
+    <t>Nước cốt dừa</t>
+  </si>
+  <si>
+    <t>Bánh tằm, Thịt</t>
+  </si>
+  <si>
+    <t>Béo</t>
+  </si>
+  <si>
+    <t>Cá, Hải sản, Bún</t>
+  </si>
+  <si>
+    <t>Mắm</t>
+  </si>
+  <si>
+    <t>Hải sản, Gạo</t>
+  </si>
+  <si>
+    <t>Rau củ quả, Dầu mè</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ngọt</t>
+  </si>
+  <si>
+    <t>Gạo, Thịt, Trứng</t>
   </si>
 </sst>
 </file>
@@ -2105,7 +2135,7 @@
         <v>23</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>294</v>
+        <v>336</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>38</v>
@@ -2137,7 +2167,7 @@
         <v>144</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>24</v>
@@ -2146,10 +2176,10 @@
         <v>309</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>310</v>
@@ -2169,19 +2199,19 @@
         <v>233</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>335</v>
+        <v>294</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>281</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>282</v>
@@ -2201,22 +2231,22 @@
         <v>82</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>294</v>
+        <v>342</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>314</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>301</v>
@@ -2227,28 +2257,28 @@
         <v>287</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>105</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>313</v>
+        <v>343</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>302</v>
@@ -2259,13 +2289,13 @@
         <v>288</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>281</v>
@@ -2274,13 +2304,13 @@
         <v>309</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>303</v>
@@ -2291,28 +2321,28 @@
         <v>289</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>312</v>
+        <v>346</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>326</v>
+        <v>347</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>304</v>
@@ -2323,28 +2353,28 @@
         <v>290</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>144</v>
+        <v>16</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>281</v>
+        <v>33</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>326</v>
+        <v>347</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>305</v>
@@ -2355,28 +2385,28 @@
         <v>291</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="G10" s="1" t="s">
-        <v>313</v>
+        <v>350</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>306</v>
@@ -2387,28 +2417,28 @@
         <v>292</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>312</v>
+        <v>346</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>331</v>
+        <v>352</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>326</v>
+        <v>353</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>307</v>
@@ -2425,19 +2455,19 @@
         <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>276</v>
+        <v>346</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>276</v>
+        <v>355</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>276</v>
+        <v>324</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>12</v>
@@ -2600,7 +2630,7 @@
         <v>276</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>39</v>
@@ -2760,7 +2790,7 @@
         <v>276</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>62</v>
@@ -3528,7 +3558,7 @@
         <v>276</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="J46" s="6" t="s">
         <v>166</v>
@@ -3910,7 +3940,7 @@
         <v>276</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="J58" s="6" t="s">
         <v>213</v>

</xml_diff>